<commit_message>
Reduser til 7 features + fiks datalekkasje i trening
Feature-sett: 13 -> 7 (ENV_MEAN, ENV_STD, WAMP, ZC, SSC, MNF, MDF).
De gamle 13 var mest duplikater (29 par med |r|>0.9). La til MNF/MDF
(mean/median frequency) som er amplitude-uavhengige og loefter
opening-vs-closing fra 62% (amplitude alene) til 90% (gruppert CV).

- process_emg.py: relative stier + 7 features (la til _mnf_mdf)
- process_features.py: FEATURE_NAVN -> 7
- feature_selection_report.py: nytt script med forsvars-figurer
- Train_deep.py: FEATURES -> 7 + GroupShuffleSplit paa opptak_id
  (datalekkasje-fiks) + retrent emg_model_deep.pt
- README.md: full dokumentasjon + synk-invarianter

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/processed/Stats/Open_close_stats/feature_stats.xlsx
+++ b/data/processed/Stats/Open_close_stats/feature_stats.xlsx
@@ -413,74 +413,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN6"/>
+  <dimension ref="A1:V6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr"/>
       <c r="B1" t="inlineStr">
         <is>
-          <t>MAV</t>
+          <t>ENV_MEAN</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>RMS</t>
+          <t>ENV_STD</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>WL</t>
+          <t>WAMP</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>VAR</t>
+          <t>ZC</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>IEMG</t>
+          <t>SSC</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>ZC</t>
+          <t>MNF</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>SSC</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>WAMP</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>PEAK</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>ENV_MEAN</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>ENV_STD</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>ENV_MAX</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
-        <is>
-          <t>ENV_RANGE</t>
+          <t>MDF</t>
         </is>
       </c>
     </row>
@@ -591,96 +561,6 @@
           <t>median</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>std</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>median</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>std</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>median</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>std</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>median</t>
-        </is>
-      </c>
-      <c r="AF2" t="inlineStr">
-        <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t>std</t>
-        </is>
-      </c>
-      <c r="AH2" t="inlineStr">
-        <is>
-          <t>median</t>
-        </is>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="AJ2" t="inlineStr">
-        <is>
-          <t>std</t>
-        </is>
-      </c>
-      <c r="AK2" t="inlineStr">
-        <is>
-          <t>median</t>
-        </is>
-      </c>
-      <c r="AL2" t="inlineStr">
-        <is>
-          <t>mean</t>
-        </is>
-      </c>
-      <c r="AM2" t="inlineStr">
-        <is>
-          <t>std</t>
-        </is>
-      </c>
-      <c r="AN2" t="inlineStr">
-        <is>
-          <t>median</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -696,121 +576,67 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5.22</v>
+        <v>516.6799999999999</v>
       </c>
       <c r="C4" t="n">
-        <v>8.69</v>
+        <v>4.99</v>
       </c>
       <c r="D4" t="n">
-        <v>2.94</v>
+        <v>514.95</v>
       </c>
       <c r="E4" t="n">
-        <v>7.18</v>
+        <v>1.3</v>
       </c>
       <c r="F4" t="n">
-        <v>14.48</v>
+        <v>4.54</v>
       </c>
       <c r="G4" t="n">
-        <v>3.68</v>
+        <v>0.4</v>
       </c>
       <c r="H4" t="n">
-        <v>173.68</v>
+        <v>2.73</v>
       </c>
       <c r="I4" t="n">
-        <v>236.22</v>
+        <v>6.02</v>
       </c>
       <c r="J4" t="n">
-        <v>104</v>
+        <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>196.59</v>
+        <v>6.61</v>
       </c>
       <c r="L4" t="n">
-        <v>1409.91</v>
+        <v>4.51</v>
       </c>
       <c r="M4" t="n">
-        <v>7.09</v>
+        <v>6</v>
       </c>
       <c r="N4" t="n">
-        <v>260.93</v>
+        <v>22.49</v>
       </c>
       <c r="O4" t="n">
-        <v>434.31</v>
+        <v>5.55</v>
       </c>
       <c r="P4" t="n">
-        <v>147</v>
+        <v>23</v>
       </c>
       <c r="Q4" t="n">
-        <v>6.61</v>
+        <v>41.04</v>
       </c>
       <c r="R4" t="n">
-        <v>4.51</v>
+        <v>8.67</v>
       </c>
       <c r="S4" t="n">
-        <v>6</v>
+        <v>41.39</v>
       </c>
       <c r="T4" t="n">
-        <v>30.71</v>
+        <v>34.09</v>
       </c>
       <c r="U4" t="n">
-        <v>4.32</v>
+        <v>11.45</v>
       </c>
       <c r="V4" t="n">
-        <v>31</v>
-      </c>
-      <c r="W4" t="n">
-        <v>2.73</v>
-      </c>
-      <c r="X4" t="n">
-        <v>6.02</v>
-      </c>
-      <c r="Y4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>20.43</v>
-      </c>
-      <c r="AA4" t="n">
-        <v>45.43</v>
-      </c>
-      <c r="AB4" t="n">
-        <v>10</v>
-      </c>
-      <c r="AC4" t="n">
-        <v>516.6799999999999</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>4.99</v>
-      </c>
-      <c r="AE4" t="n">
-        <v>514.95</v>
-      </c>
-      <c r="AF4" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="AG4" t="n">
-        <v>4.54</v>
-      </c>
-      <c r="AH4" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AI4" t="n">
-        <v>519.35</v>
-      </c>
-      <c r="AJ4" t="n">
-        <v>13.84</v>
-      </c>
-      <c r="AK4" t="n">
-        <v>515.7</v>
-      </c>
-      <c r="AL4" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="AM4" t="n">
-        <v>13.36</v>
-      </c>
-      <c r="AN4" t="n">
-        <v>1.43</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5">
@@ -820,121 +646,67 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>30.34</v>
+        <v>544.5599999999999</v>
       </c>
       <c r="C5" t="n">
-        <v>13.16</v>
+        <v>11.81</v>
       </c>
       <c r="D5" t="n">
-        <v>26.46</v>
+        <v>542.37</v>
       </c>
       <c r="E5" t="n">
-        <v>39</v>
+        <v>8.41</v>
       </c>
       <c r="F5" t="n">
-        <v>19.07</v>
+        <v>7.02</v>
       </c>
       <c r="G5" t="n">
-        <v>32.99</v>
+        <v>5.88</v>
       </c>
       <c r="H5" t="n">
-        <v>1044.7</v>
+        <v>30.04</v>
       </c>
       <c r="I5" t="n">
-        <v>430.83</v>
+        <v>7.92</v>
       </c>
       <c r="J5" t="n">
-        <v>1009.5</v>
+        <v>31.5</v>
       </c>
       <c r="K5" t="n">
-        <v>1681.11</v>
+        <v>10.02</v>
       </c>
       <c r="L5" t="n">
-        <v>1864.17</v>
+        <v>3.67</v>
       </c>
       <c r="M5" t="n">
-        <v>1004.05</v>
+        <v>10</v>
       </c>
       <c r="N5" t="n">
-        <v>1516.79</v>
+        <v>15.82</v>
       </c>
       <c r="O5" t="n">
-        <v>657.89</v>
+        <v>5.37</v>
       </c>
       <c r="P5" t="n">
-        <v>1323</v>
+        <v>16</v>
       </c>
       <c r="Q5" t="n">
-        <v>10.02</v>
+        <v>31.77</v>
       </c>
       <c r="R5" t="n">
-        <v>3.67</v>
+        <v>7.95</v>
       </c>
       <c r="S5" t="n">
-        <v>10</v>
+        <v>31.7</v>
       </c>
       <c r="T5" t="n">
-        <v>24.17</v>
+        <v>24.16</v>
       </c>
       <c r="U5" t="n">
-        <v>3.36</v>
+        <v>10.44</v>
       </c>
       <c r="V5" t="n">
-        <v>24</v>
-      </c>
-      <c r="W5" t="n">
-        <v>30.04</v>
-      </c>
-      <c r="X5" t="n">
-        <v>7.92</v>
-      </c>
-      <c r="Y5" t="n">
-        <v>31.5</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>106.4</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>64.38</v>
-      </c>
-      <c r="AB5" t="n">
-        <v>88.5</v>
-      </c>
-      <c r="AC5" t="n">
-        <v>544.5599999999999</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>11.81</v>
-      </c>
-      <c r="AE5" t="n">
-        <v>542.37</v>
-      </c>
-      <c r="AF5" t="n">
-        <v>8.41</v>
-      </c>
-      <c r="AG5" t="n">
-        <v>7.02</v>
-      </c>
-      <c r="AH5" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="AI5" t="n">
-        <v>558.54</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>20.2</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>553.4</v>
-      </c>
-      <c r="AL5" t="n">
-        <v>27.24</v>
-      </c>
-      <c r="AM5" t="n">
-        <v>19.91</v>
-      </c>
-      <c r="AN5" t="n">
-        <v>20.32</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
@@ -944,133 +716,73 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>50.32</v>
+        <v>566.21</v>
       </c>
       <c r="C6" t="n">
-        <v>30.99</v>
+        <v>28.67</v>
       </c>
       <c r="D6" t="n">
-        <v>42.71</v>
+        <v>558.4</v>
       </c>
       <c r="E6" t="n">
-        <v>62.09</v>
+        <v>15.54</v>
       </c>
       <c r="F6" t="n">
-        <v>43.17</v>
+        <v>17.64</v>
       </c>
       <c r="G6" t="n">
-        <v>48.66</v>
+        <v>6.49</v>
       </c>
       <c r="H6" t="n">
-        <v>1603.59</v>
+        <v>30.6</v>
       </c>
       <c r="I6" t="n">
-        <v>1197.13</v>
+        <v>12.72</v>
       </c>
       <c r="J6" t="n">
-        <v>1168</v>
+        <v>33</v>
       </c>
       <c r="K6" t="n">
-        <v>4293.33</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="L6" t="n">
-        <v>7185.29</v>
+        <v>5.12</v>
       </c>
       <c r="M6" t="n">
-        <v>864.61</v>
+        <v>9</v>
       </c>
       <c r="N6" t="n">
-        <v>2516</v>
+        <v>15.14</v>
       </c>
       <c r="O6" t="n">
-        <v>1549.44</v>
+        <v>5.91</v>
       </c>
       <c r="P6" t="n">
-        <v>2135.5</v>
+        <v>16</v>
       </c>
       <c r="Q6" t="n">
-        <v>8.699999999999999</v>
+        <v>37.89</v>
       </c>
       <c r="R6" t="n">
-        <v>5.12</v>
+        <v>10.16</v>
       </c>
       <c r="S6" t="n">
-        <v>9</v>
+        <v>39.99</v>
       </c>
       <c r="T6" t="n">
-        <v>23.81</v>
+        <v>32.73</v>
       </c>
       <c r="U6" t="n">
-        <v>3.5</v>
+        <v>12.81</v>
       </c>
       <c r="V6" t="n">
-        <v>24</v>
-      </c>
-      <c r="W6" t="n">
-        <v>30.6</v>
-      </c>
-      <c r="X6" t="n">
-        <v>12.72</v>
-      </c>
-      <c r="Y6" t="n">
-        <v>33</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>149.08</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>125.47</v>
-      </c>
-      <c r="AB6" t="n">
-        <v>97</v>
-      </c>
-      <c r="AC6" t="n">
-        <v>566.21</v>
-      </c>
-      <c r="AD6" t="n">
-        <v>28.67</v>
-      </c>
-      <c r="AE6" t="n">
-        <v>558.4</v>
-      </c>
-      <c r="AF6" t="n">
-        <v>15.54</v>
-      </c>
-      <c r="AG6" t="n">
-        <v>17.64</v>
-      </c>
-      <c r="AH6" t="n">
-        <v>6.49</v>
-      </c>
-      <c r="AI6" t="n">
-        <v>591.63</v>
-      </c>
-      <c r="AJ6" t="n">
-        <v>51.27</v>
-      </c>
-      <c r="AK6" t="n">
-        <v>568.78</v>
-      </c>
-      <c r="AL6" t="n">
-        <v>48.9</v>
-      </c>
-      <c r="AM6" t="n">
-        <v>49.94</v>
-      </c>
-      <c r="AN6" t="n">
-        <v>22.62</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="7">
     <mergeCell ref="H1:J1"/>
-    <mergeCell ref="Z1:AB1"/>
-    <mergeCell ref="AC1:AE1"/>
-    <mergeCell ref="AF1:AH1"/>
     <mergeCell ref="T1:V1"/>
-    <mergeCell ref="AI1:AK1"/>
-    <mergeCell ref="W1:Y1"/>
-    <mergeCell ref="AL1:AN1"/>
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="N1:P1"/>
     <mergeCell ref="Q1:S1"/>

</xml_diff>